<commit_message>
Adiciona campanha de doacao, acervo de arquivos e adaptacao a telas estreitas
</commit_message>
<xml_diff>
--- a/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
+++ b/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Divergências TCC1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"CRÍTICA")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"CRÍTICA")</f>
         <v/>
       </c>
     </row>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"ESSENCIAL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"ESSENCIAL")</f>
         <v/>
       </c>
     </row>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"IMPORTANTE")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"IMPORTANTE")</f>
         <v/>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"DESEJÁVEL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"DESEJÁVEL")</f>
         <v/>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTA('Requisitos Funcionais'!B2:B81)</f>
+        <f>COUNTA('Requisitos Funcionais'!B2:B86)</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3213,32 +3213,32 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>RF-PAI-001</t>
+          <t>RF-VOL-014</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Painel de quem conduz a turma</t>
+          <t>Publicar campanha de doação</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
+          <t>A organização cadastra uma arrecadação de itens, como agasalhos ou alimentos, definindo como a contribuição será contada.</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
+          <t>Modalidade da oportunidade. A unidade é texto livre — peças de agasalho, quilos de alimento — porque qualquer lista fixa não teria a categoria da próxima campanha. Meta é opcional. Vagas e carga horária não se aplicam: campanha não limita participantes nem cumpre hora.</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
@@ -3253,32 +3253,32 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>RF-PAI-002</t>
+          <t>RF-VOL-015</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Painel da organização parceira</t>
+          <t>Declarar doação</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
+          <t>Estudante informa quanto pretende entregar à campanha.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
+          <t>POST em inscrever, com quantidade declarada e descrição opcional do item. É declaração de intenção: o valor fica registrado à parte e não entra na contagem da campanha até a organização confirmar o recebimento.</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H67" s="9" t="inlineStr">
@@ -3293,37 +3293,37 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-001</t>
+          <t>RF-VOL-016</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Entregar notificação em tempo real</t>
+          <t>Confirmar recebimento da doação</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>O aviso chega sem recarregar a página.</t>
+          <t>A organização registra quanto de fato recebeu, que pode divergir do que foi declarado.</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
+          <t>POST em concluir, com a quantidade confirmada. Sem valor informado, vale o declarado. O campo é somente leitura para o estudante: se ele pudesse registrar o próprio recebimento, o total da campanha deixaria de significar algo. Emite o certificado na mesma operação.</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3333,27 +3333,27 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-002</t>
+          <t>RF-VOL-017</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Listar notificações</t>
+          <t>Acompanhar a arrecadação</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
+          <t>A página da campanha mostra quanto já foi arrecadado e, havendo meta, o progresso em relação a ela.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
+          <t>Soma apenas as quantidades confirmadas em participações concluídas. Sem meta declarada não há barra de progresso: a barra precisa de um denominador, e inventar um faria a campanha parecer mais adiantada do que está.</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
@@ -3373,37 +3373,37 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-003</t>
+          <t>RF-VOL-018</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Marcar notificação como lida</t>
+          <t>Certificar participação em campanha</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>Usuário marca um aviso ou todos de uma vez.</t>
+          <t>Quem doou recebe certificado declarando a contribuição.</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
+          <t>O texto do certificado muda com a modalidade: registra o que foi entregue e acrescenta que a organização atribui àquela participação o equivalente a um número de horas por ela definido. A formulação é deliberada — doar não é cumprir hora, e quem receber o documento precisa saber que avalia uma equivalência declarada pela entidade.</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3413,37 +3413,37 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-004</t>
+          <t>RF-PAI-001</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Limpar notificações</t>
+          <t>Painel de quem conduz a turma</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Usuário descarta os avisos já lidos.</t>
+          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/limpar/.</t>
+          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>DESEJÁVEL</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3453,37 +3453,37 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-005</t>
+          <t>RF-PAI-002</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Agrupar aviso por conversa</t>
+          <t>Painel da organização parceira</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
+          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
+          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3493,32 +3493,32 @@
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>RF-PRF-001</t>
+          <t>RF-NOT-001</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Visualizar perfil</t>
+          <t>Entregar notificação em tempo real</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
+          <t>O aviso chega sem recarregar a página.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
+          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -3533,27 +3533,27 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>RF-PRF-002</t>
+          <t>RF-NOT-002</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Consultar histórico de participação</t>
+          <t>Listar notificações</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
+          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
+          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3573,37 +3573,37 @@
       </c>
       <c r="B75" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-001</t>
+          <t>RF-NOT-003</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Acompanhar o curso por disciplina</t>
+          <t>Marcar notificação como lida</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
+          <t>Usuário marca um aviso ou todos de uma vez.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
+          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3613,37 +3613,37 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>RF-COO-002</t>
+          <t>RF-NOT-004</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Detalhar uma disciplina</t>
+          <t>Limpar notificações</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+          <t>Usuário descarta os avisos já lidos.</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+          <t>POST /api/notificacoes/limpar/.</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -3653,32 +3653,32 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-003</t>
+          <t>RF-NOT-005</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Importar a matriz curricular</t>
+          <t>Agrupar aviso por conversa</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H77" s="9" t="inlineStr">
@@ -3693,37 +3693,37 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>RF-AUD-001</t>
+          <t>RF-PRF-001</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Registrar ações sensíveis</t>
+          <t>Visualizar perfil</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Perfil</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3733,27 +3733,27 @@
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>RF-SIS-001</t>
+          <t>RF-PRF-002</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Alternar entre tema claro e escuro</t>
+          <t>Consultar histórico de participação</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Perfil</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
+          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
+          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
@@ -3773,37 +3773,37 @@
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>RF-SIS-002</t>
+          <t>RF-COO-001</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Consultar a documentação da API</t>
+          <t>Acompanhar o curso por disciplina</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>A especificação da API fica acessível e navegável.</t>
+          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3813,42 +3813,242 @@
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
+          <t>RF-COO-002</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>Detalhar uma disciplina</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>RF-COO-003</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Importar a matriz curricular</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>RF-AUD-001</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>Registrar ações sensíveis</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+        </is>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>RF-SIS-001</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Alternar entre tema claro e escuro</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>RF-SIS-002</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>Consultar a documentação da API</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>A especificação da API fica acessível e navegável.</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
           <t>RF-SIS-003</t>
         </is>
       </c>
-      <c r="C81" s="9" t="inlineStr">
+      <c r="C86" s="8" t="inlineStr">
         <is>
           <t>Carregar dados de demonstração</t>
         </is>
       </c>
-      <c r="D81" s="9" t="inlineStr">
+      <c r="D86" s="8" t="inlineStr">
         <is>
           <t>Sistema</t>
         </is>
       </c>
-      <c r="E81" s="9" t="inlineStr">
+      <c r="E86" s="8" t="inlineStr">
         <is>
           <t>A plataforma pode ser povoada com um semestre completo para demonstração e avaliação.</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
+      <c r="F86" s="8" t="inlineStr">
         <is>
           <t>Comando popular_demonstracao, com semente fixa para que a mesma execução produza sempre o mesmo conjunto. Gera disciplinas com ritmos distintos de atividade, deliberadamente incluindo uma sem professor atribuído, para que o painel de coordenação tenha o que apontar.</t>
         </is>
       </c>
-      <c r="G81" s="9" t="inlineStr">
+      <c r="G86" s="8" t="inlineStr">
         <is>
           <t>Coordenação</t>
         </is>
       </c>
-      <c r="H81" s="9" t="inlineStr">
+      <c r="H86" s="8" t="inlineStr">
         <is>
           <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H81"/>
+  <autoFilter ref="A1:H86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3859,7 +4059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4002,12 +4202,12 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Registro de doações e pontuação por item</t>
+          <t>Registro de doações</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Removido</t>
+          <t>Reformulado</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -4017,7 +4217,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Removido junto com o sistema de pontuação, pelo mesmo motivo.</t>
+          <t>O TCC1 previa doação como gerador de pontos, com fórmula progressiva por item. A pontuação foi removida, mas a doação em si retornou como modalidade própria de oportunidade: a organização publica uma campanha, define a unidade de contagem e uma meta opcional, e o estudante declara o que pretende entregar. O que mudou foi o propósito — antes o item valia pontos numa classificação, agora ele conta para uma arrecadação com destino concreto.</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4227,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Restrição de publicação por decisão pedagógica</t>
+          <t>Separação entre doação declarada e confirmada</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -4037,12 +4237,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>RF-FOR-015</t>
+          <t>Sem correspondência no TCC1</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Não estava previsto. Surgiu da distinção entre conteúdo que infringe regra, que é caso de denúncia, e resposta que entrega o exercício pronto, que não infringe nada e ainda assim prejudica a turma.</t>
+          <t>O desenho original registrava a doação num único valor. Na implementação ficou claro que intenção e recebimento são coisas distintas: somar o que os estudantes prometeram faria a campanha exibir uma arrecadação que nunca chegou. A confirmação passou a ser ato exclusivo da organização.</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4252,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Acervo de arquivos por disciplina</t>
+          <t>Restrição de publicação por decisão pedagógica</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -4062,12 +4262,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-014</t>
+          <t>RF-FOR-015</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Não estava previsto. Surgiu do uso: o material chegava por três caminhos diferentes e reencontrá-lo exigia lembrar por qual deles havia passado.</t>
+          <t>Não estava previsto. Surgiu da distinção entre conteúdo que infringe regra, que é caso de denúncia, e resposta que entrega o exercício pronto, que não infringe nada e ainda assim prejudica a turma.</t>
         </is>
       </c>
     </row>
@@ -4077,27 +4277,52 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
+          <t>Acervo de arquivos por disciplina</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Incorporado</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>RF-COL-014</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Não estava previsto. Surgiu do uso: o material chegava por três caminhos diferentes e reencontrá-lo exigia lembrar por qual deles havia passado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
           <t>Certificado com assinatura digital X.509</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Reduzido</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>RF-VOL-012 do TCC1</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>O certificado é emitido em PDF com código único de conferência. A assinatura criptográfica com certificado digital exigiria infraestrutura de chaves institucional, fora do alcance do trabalho.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>